<commit_message>
Date context for 19 1939-40 lists (1931 statement, 1936 union meetings, etc.); China Handbook interim
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MKgSdDvVSCL7zgQ1r4fLnk
</commit_message>
<xml_diff>
--- a/downloads/japan-1910-tables.xlsx
+++ b/downloads/japan-1910-tables.xlsx
@@ -35,6 +35,14 @@
     <sheet name="p0083_4" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="p0083_5" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="p0084_1" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="p0085_1" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="p0086_1" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="p0086_2" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="p0086_3" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="p0091_1" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="p0091_2" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="p0092_1" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="p0092_2" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,9 +51,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -91,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,6 +115,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1251,6 +1261,222 @@
       <c r="E32" t="inlineStr">
         <is>
           <t>https://archive.org/details/japan-year-book-1910/page/n84/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>p0085_1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Foreigners Residing in Japan</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>18, 19</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n85/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>p0086_1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Foreigners in Japan by Districts</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n86/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>p0086_2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Foreigners in Japan by Nationality</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n86/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>p0086_3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Ainu in Hokkaido</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n86/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>p0091_1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Holders of the Grand Order</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n91/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>p0091_2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Holders of the 1st Grade Golden Kite</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n91/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>p0092_1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Holders of Decorations</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n92/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>p0092_2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Holders of the Golden Kite Military Honour</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n92/mode/1up</t>
         </is>
       </c>
     </row>
@@ -1283,6 +1509,14 @@
     <hyperlink ref="A30" location="'p0083_4'!A1"/>
     <hyperlink ref="A31" location="'p0083_5'!A1"/>
     <hyperlink ref="A32" location="'p0084_1'!A1"/>
+    <hyperlink ref="A33" location="'p0085_1'!A1"/>
+    <hyperlink ref="A34" location="'p0086_1'!A1"/>
+    <hyperlink ref="A35" location="'p0086_2'!A1"/>
+    <hyperlink ref="A36" location="'p0086_3'!A1"/>
+    <hyperlink ref="A37" location="'p0091_1'!A1"/>
+    <hyperlink ref="A38" location="'p0091_2'!A1"/>
+    <hyperlink ref="A39" location="'p0092_1'!A1"/>
+    <hyperlink ref="A40" location="'p0092_2'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9849,7 +10083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D110"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -11424,9 +11658,342 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Male+Female=Total by row: does NOT reconcile for Harbin (292+325=617 vs 627), Vladivostock (1,365+836=2,201 vs 2,203), 1904 (117,715+36,921=154,636 vs 148,636); re-read, confirmed as printed. All other complete rows reconcile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Indented city rows are selected places, not exhaustive sub-divisions, so country figures exceed their sums (checks below are informational).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>China (first line) = Peking…Antung non-* lines: Male 19,235 vs parts 12,764 does NOT reconcile (diff +6,471); Female: not checkable (blank cell); Total 33,112 vs parts 21,325 does NOT reconcile (diff +11,787)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>China * line = Fuchow*+Amoy*: Male *1,609 vs parts 1,495 does NOT reconcile (diff +114); Female 284 vs parts 266 does NOT reconcile (diff +18); Total 1,893 vs parts 1,761 does NOT reconcile (diff +132)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Siberia = Harbin…Vladivostock: Male 2,580 vs parts 1,884 does NOT reconcile (diff +696); Female 2,376 vs parts 1,470 does NOT reconcile (diff +906); Total 4,956 vs parts 3,366 does NOT reconcile (diff +1,590)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>British Asia = Hongkong+Singapore+Calcutta: Male 1,095 vs parts 872 does NOT reconcile (diff +223); Female 1,838 vs parts 1,302 does NOT reconcile (diff +536); Total: not checkable (blank cell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Asia Total = China+Siberia+Siam+British Asia+Amoy(2nd): Male 69,957 vs parts 23,029 does NOT reconcile (diff +46,928); Female: not checkable (blank cell); Total 121,943 vs parts 41,189 does NOT reconcile (diff +80,754)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Asia Total * line = China*+Siam*: Male *1,620 vs parts 1,620 reconciles; Female 284 vs parts 284 reconciles; Total 1,904 vs parts 1,904 reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Europe Total = England…Russia (countries): Male 608 vs parts 608 reconciles; Female 86 vs parts 86 reconciles; Total 694 vs parts 694 reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>America Total = U.S.A.+Canada+Mexico: Male 27,189 vs parts 27,189 reconciles; Female 2,796 vs parts 2,796 reconciles; Total 29,985 vs parts 29,985 reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>U.S.A. = Illinois…Alaska: Male 18,546 vs parts 7,645 does NOT reconcile (diff +10,901); Female 1,534 vs parts 990 does NOT reconcile (diff +544); Total 20,080 vs parts 8,635 does NOT reconcile (diff +11,445)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>South America Total = Brazil+Argentine+Peru: Male 2,151 vs parts 2,151 reconciles; Female 111 vs parts 111 reconciles; Total 2,262 vs parts 2,262 reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Oceania Total = Oceania (U.S.A.)+Do. (British)+Do. (German): Male: not checkable (blank cell); Female 20,213 vs parts 20,213 reconciles; Total 77,336 vs parts 77,336 reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Grand Total = section Totals: Male: not checkable (blank cell); Female 75,192 vs parts 75,192 reconciles; Total 232,220 vs parts 232,220 reconciles</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Foreigners Residing in Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Population · printed pp. 18, 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n85/mode/1up, https://archive.org/details/japan-year-book-1910/page/n86/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>At end of</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Males</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Females</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>1902</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>10318</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>3939</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>14257</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>1903</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>9903</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>3806</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>13706</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>1904</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>11569</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>3928</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>15497</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>1905</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>12573</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>3985</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>16558</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>1906</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>14485</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>4489</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>18972</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>1907</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>14561</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>4347</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>18908</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1902: Males+Females=14,257 vs Total 14,257 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1903: Males+Females=13,709 vs Total 13,706 — does NOT reconcile (diff -3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1904: Males+Females=15,497 vs Total 15,497 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1905: Males+Females=16,558 vs Total 16,558 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1906: Males+Females=18,974 vs Total 18,972 — does NOT reconcile (diff -2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1907: Males+Females=18,908 vs Total 18,908 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rows 1906-1907 printed at top of p. 19 (leaf p0086). 1903 row re-read; confirmed as printed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11709,6 +12276,2923 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Foreigners in Japan by Districts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Population · printed pp. 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Official returns put the number of foreign residents in Japan from the end of 1904 to 1907 as follows:—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n86/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Districts</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>1904</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>1905</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>1906</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>1907 — Males</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>1907 — Females</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>1907 — Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>3240</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>4232</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>5555</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>4745</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>232</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>4977</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kanagawa</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>5541</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>5745</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>6088</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>4276</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>2046</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>6322</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Aichi</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Miyagi</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>78</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kyoto</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>141</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>101</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>578</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>719</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>577</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hyogo</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>3294</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>3222</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>3727</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>2733</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>1148</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>3881</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Hiroshima</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Yamaguchi</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Nagasaki</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>1579</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>1553</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>1109</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>414</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>1523</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fukuoka</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>111</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>243</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hokkaido</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>212</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>234</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>243</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>No total row printed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1907 Males+Females=Total: all rows reconcile</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Foreigners in Japan by Nationality</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Population · printed pp. 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nationality of foreigners numbering 100 or above is:—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n86/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Nationality</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>1905</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>1906</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>1907 — Male</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>1907 — Female</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>1907 — Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>10388</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>12425</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>10239</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>2034</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>12273</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>British</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>2114</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>2155</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>1442</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>851</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>2293</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Americans</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>1612</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>1650</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>931</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>693</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>1624</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Germans</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>616</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>670</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>476</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Frenchmen</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>531</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>540</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>309</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Koreans</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>303</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>254</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>452</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Russians</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>211</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>113</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Portuguese</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>114</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>83</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Total (inc. others)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" s="12" t="n">
+        <v>14.561</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>4347</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>18908</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Total line printed as prose: 'Total (inc. others) 14.561 Males 4,347 Females 18,908 Total.' (with a point in 14.561); includes nationalities not listed, so parts are not expected to sum to it. Nothing printed for 1905/1906 in the total line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1907 Male+Female=Total: all rows reconcile</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Heading printed 'Natonality.' (sic).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Ainu in Hokkaido</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Population · printed pp. 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n86/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>At end of</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>1905</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>8598</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>9034</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>19632</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>1906</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>8528</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>8914</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>17442</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>1907</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>8690</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>9025</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>17715</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Inc. or Dec.</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>+162</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>+111</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>+273</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>In 1907 the birthrates and deathrates were as follows:—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[Item]</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Birth</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" s="9" t="n">
+        <v>242</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>226</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1905: Male+Female=17,632 vs Total 19,632 — does NOT reconcile (diff +2,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1906: Male+Female=17,442 vs Total 17,442 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1907: Male+Female=17,715 vs Total 17,715 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Inc. or Dec.: Male+Female=273 vs Total +273 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Inc. or Dec. vs 1907 minus 1906: Male +162, Female +111, Total +273 — Male and Female match printed +162/+111; Total matches +273.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Part B row Birth, col Male: printed '2?0', middle digit broken; left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Death: 227+226=453 — reconciles.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Holders of the Grand Order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n91/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Rank and Office</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Yamagata</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Marshal, Prince (with Collar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oyama</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>" " "</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Matsukata</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Marquis, Privy Councillor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Inouye</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Marquis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tokudaiji</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Marquis, Grand Chamberlain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Katsura</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Marquis, General.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Togo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Count, full-Admiral; Chief, Naval Staff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Names printed in italics, each followed by a comma and leader dots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Oyama: three ditto marks under 'Marshal, Prince (with Collar)'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>'Matsukata' and 'Katsura' have a broken 't'/'s' in the scan.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Holders of the 1st Grade Golden Kite</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n91/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Rank and Office</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hasejawa</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Visc., General.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Iju-in</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Baron, Vice Admiral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ito</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Count, Admiral of the Fleet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kamimura</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Baron Vice-Adm., Com. of Yokosuka Admiralty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kataoka</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Baron Admiral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kawamura</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Visc., General.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Nishi</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Visc., General.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Noji</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Count, General.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Oka</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Count, General.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Oyama</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Prince, Marshal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Terauchi</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Visc., Gen., Minister of War.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Togo</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Count, Admiral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Yamagata</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Prince, Marshal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Yamamoto</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Count, Admiral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Names printed in italics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>'Hasejawa' as it appears in print (italic g/j; probably Hasegawa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>'Yamamoto' has a broken 't' in the scan.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Holders of Decorations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n92/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>G.O. — C.C.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>G.O. — G.C.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>1st Class — R.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>1st Class — R.S.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>1st Class — S.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>1st Class — C.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>2nd Class — R.S.</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>2nd Class — S.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>2nd Class — C.</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>3rd Class — R.S.</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>3rd Class — S.</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>3rd Class — C.</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>4th Class — R.S.</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>4th Class — S.</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>4th Class — C.</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>5th Class — R.S.</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>5th Class — S.</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>5th Class — C.</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>6th Class — R.S.</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>6th Class — S.</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>6th Class — C.</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>7th Class — R.S.</t>
+        </is>
+      </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>7th Class — S.</t>
+        </is>
+      </c>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>7th Class — C.</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>8th Class — R.S.</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>8th Class — S.</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="inlineStr">
+        <is>
+          <t>8th Class — C.</t>
+        </is>
+      </c>
+      <c r="AC6" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>1902</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>163</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="R7" s="8" t="n">
+        <v>1141</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T7" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="U7" s="9" t="n">
+        <v>561</v>
+      </c>
+      <c r="V7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="X7" s="8" t="n">
+        <v>2352</v>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" s="9" t="n">
+        <v>119</v>
+      </c>
+      <c r="AA7" s="9" t="n">
+        <v>758</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>1903</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>137</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="R8" s="9" t="n">
+        <v>808</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T8" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="U8" s="9" t="n">
+        <v>370</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="X8" s="8" t="n">
+        <v>1455</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z8" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="AA8" s="9" t="n">
+        <v>942</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC8" s="8" t="n">
+        <v>3914</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>1904</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="O9" s="9" t="n">
+        <v>229</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="n">
+        <v>216</v>
+      </c>
+      <c r="R9" s="9" t="n">
+        <v>381</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T9" s="9" t="n">
+        <v>660</v>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W9" s="9" t="n">
+        <v>351</v>
+      </c>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z9" s="9" t="n">
+        <v>934</v>
+      </c>
+      <c r="AA9" s="8" t="n">
+        <v>1579</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>1905</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>204</v>
+      </c>
+      <c r="O10" s="9" t="n">
+        <v>655</v>
+      </c>
+      <c r="P10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="R10" s="9" t="n">
+        <v>554</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T10" s="8" t="n">
+        <v>1082</v>
+      </c>
+      <c r="U10" s="8" t="n">
+        <v>1537</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W10" s="8" t="n">
+        <v>5278</v>
+      </c>
+      <c r="X10" s="8" t="n">
+        <v>1764</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z10" s="8" t="n">
+        <v>21692</v>
+      </c>
+      <c r="AA10" s="8" t="n">
+        <v>3144</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC10" s="8" t="n">
+        <v>36357</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>1906</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>117</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>989</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>3474</v>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>107</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q11" s="8" t="n">
+        <v>13340</v>
+      </c>
+      <c r="R11" s="9" t="n">
+        <v>249</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T11" s="8" t="n">
+        <v>86782</v>
+      </c>
+      <c r="U11" s="8" t="n">
+        <v>3002</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W11" s="8" t="n">
+        <v>94260</v>
+      </c>
+      <c r="X11" s="8" t="n">
+        <v>14422</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z11" s="8" t="n">
+        <v>529388</v>
+      </c>
+      <c r="AA11" s="8" t="n">
+        <v>235268</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC11" s="8" t="n">
+        <v>981461</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>1907</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>131</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>143</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>910</v>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>1123</v>
+      </c>
+      <c r="R12" s="9" t="n">
+        <v>480</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>1838</v>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>2478</v>
+      </c>
+      <c r="V12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" s="8" t="n">
+        <v>3650</v>
+      </c>
+      <c r="X12" s="8" t="n">
+        <v>2881</v>
+      </c>
+      <c r="Y12" s="9" t="n">
+        <v>212</v>
+      </c>
+      <c r="Z12" s="8" t="n">
+        <v>10244</v>
+      </c>
+      <c r="AA12" s="8" t="n">
+        <v>11522</v>
+      </c>
+      <c r="AB12" s="8" t="n">
+        <v>1742</v>
+      </c>
+      <c r="AC12" s="8" t="n">
+        <v>37602</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Footnotes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Notes:—G.O. Grand Order. C.C. Crysan'mum Collar. G.C. Grand Corden Cry'mum. R. Rising Sun and Paulonia. R.S Rising Sun. S. Sacred Treasury. C. Crown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Printed rotated (landscape) on the page. Print is very small and bold; 3/8 and 5/6 are hard to tell apart in this scan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Blank (ambiguous glyphs): 1903 'G.O. — G.C.' and '1st Class — R.' (each 3 or 8); 1906 '1st Class — R.S.' (printed '?0', first digit 3 or 8); 1902 '7th Class — C.' (5 or 6); 1902 Total (first digit 5 or 6: '?,391'); 1904 '6th Class — S.' ('?56', first digit 5 or 6); 1904 '7th Class — S.' ('?88', first digit 5 or 6); 1904 Total ('?,862', first digit 5 or 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1902: row total not checkable (blank cell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1903: row total not checkable (blank cell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1904: row total not checkable (blank cell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1905: printed Total 36,357, parts sum to 36,353 — does NOT reconcile (diff +4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1906: row total not checkable (blank cell)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1907: printed Total 37,602, parts sum to 37,592 — does NOT reconcile (diff +10)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Holders of the Golden Kite Military Honour</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n92/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>1st Merit</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>4th</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>7th</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>189[illegible]</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>1901</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>1904</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>108</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>814</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" s="8" t="n">
+        <v>1285</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>2316</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>1905</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>853</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" s="8" t="n">
+        <v>26497</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>27649</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>1906</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>1632</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>1837</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>3358</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>66533</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>73810</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>1907</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>1037</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>437</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" s="8" t="n">
+        <v>3569</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>3728</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>95443</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>105128</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Footnotes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>The annuities given in 1907 totalled yen 9,063,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Printed rotated (landscape) on the page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Row 1 year label printed '189?', last digit broken; marked [illegible].</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Row 1904, col 6th: printed '?9', first digit damaged; left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Total row, col 4th: printed '1,85?', last digit damaged; left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>189[illegible]: Total 5, parts 5 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1901: Total 188, parts 188 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1904: row not checkable</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1906: Total 73,810, parts 73,810 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1907: Total 1,160, parts 1,160 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Column 1st Merit: Total 17, parts 17 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Column 2nd: Total 76, parts 76 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Column 3rd: Total 437, parts 437 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Column 4th: not checkable</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Column 5th: Total 3,569, parts 3,569 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Column 6th: not checkable</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Column 7th: Total 95,443, parts 95,443 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Column Total: Total 105,128, parts 105,128 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Row 1905, col 6th: printed '2?2', middle digit faint/broken; left blank. 1905 row therefore not checkable.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge Japan 1910 interim; rebuild (China Handbook interim)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MKgSdDvVSCL7zgQ1r4fLnk
</commit_message>
<xml_diff>
--- a/downloads/japan-1910-tables.xlsx
+++ b/downloads/japan-1910-tables.xlsx
@@ -43,6 +43,12 @@
     <sheet name="p0091_2" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="p0092_1" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="p0092_2" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="p0093_1" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="p0093_2" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="p0094_1" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="p0094_2" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="p0094_3" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="p0095_1" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1477,6 +1483,168 @@
       <c r="E40" t="inlineStr">
         <is>
           <t>https://archive.org/details/japan-year-book-1910/page/n92/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>p0093_1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>[Number of Peers] (The Peerage and Ranks)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n93/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>p0093_2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>List of Princes</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n93/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>p0094_1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>List of Marquises</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n94/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>p0094_2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Precedent at Court According to Rank</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n94/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>p0094_3</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Principal Officials of the Imperial Household Dept.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>27, 28</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n94/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>p0095_1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Imperial Court</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Court Ladies</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/japan-year-book-1910/page/n95/mode/1up</t>
         </is>
       </c>
     </row>
@@ -1517,6 +1685,12 @@
     <hyperlink ref="A38" location="'p0091_2'!A1"/>
     <hyperlink ref="A39" location="'p0092_1'!A1"/>
     <hyperlink ref="A40" location="'p0092_2'!A1"/>
+    <hyperlink ref="A41" location="'p0093_1'!A1"/>
+    <hyperlink ref="A42" location="'p0093_2'!A1"/>
+    <hyperlink ref="A43" location="'p0094_1'!A1"/>
+    <hyperlink ref="A44" location="'p0094_2'!A1"/>
+    <hyperlink ref="A45" location="'p0094_3'!A1"/>
+    <hyperlink ref="A46" location="'p0095_1'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15198,6 +15372,897 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>[Number of Peers] (The Peerage and Ranks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>The number of Peers and its movement are shown in the following list:—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n93/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Prince</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Marquis</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Viscount</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Baron</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>1902</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>362</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>290</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>1903</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>362</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>290</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>1904</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>363</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>289</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>1905</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>362</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>291</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>1906</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>363</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>304</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>1907</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>375</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>376</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1902: Total 789, parts 789 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1903: Total 789, parts 789 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1904: Total 789, parts 789 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1905: Total 790, parts 790 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1906: Total 804, parts 803 — does NOT reconcile (diff +1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1907: Total 902, parts 902 — reconciles</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Headings printed 'Connt.' and 'Visconnt.' (broken u).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>List of Princes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>(For life see Chap. Who's Who).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n93/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ichijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ito</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Iwakura</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Konoye</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kujo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mōri</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Nijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Oyama</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sanjo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Shimazu (main house)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>" (scion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Takatsukasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tokugawa (main house)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tokugawa (last of Shoguns)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Yamagata</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Printed in two columns; left column (Ichijo … Oyama) then right column (Sanjo … Yamagata).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>'" (scion)' = ditto mark under Shimazu.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>List of Marquises</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>(For life see Chap. Who's Who)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n94/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Asano</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Daigo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hachisuka</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Hirohata</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hosokawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ikeda (Bizen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ikeda (Inaba)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Inouye</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Katsura</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Kazan-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Kido</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Kikutei</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Kuga</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Kuroda</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mayeda</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Matsudaira</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Matsukata</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nabeshima</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nakamikado</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Nakayama</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nozu</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Okubo</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Oimikado</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Saga</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Saigo (son of elder Saigo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Saigo (son of junior Saigo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Saionji</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sasaki (cr. '09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Satake</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Shijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sho</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Tokudaiji</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Tokugawa (house of Kishu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>" ( " " Mito)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>" ( " " Owari)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Yamanouchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Printed in two columns; left column (Asano … Nabeshima) then right column (Nakamikado … Yamanouchi).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ditto rows under 'Tokugawa (house of Kishu)' printed as '" ( " " Mito)' and '" ( " " Owari)'.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -15542,6 +16607,1177 @@
       <c r="A36" t="inlineStr">
         <is>
           <t>Rows 1-18 on p. 1, rows 19-23 on p. 2. No total printed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Precedent at Court According to Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n94/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Rank (in order of precedence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Holders of the Grand Order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Prime Minister.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ministers of State.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>President of the Privy Council.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Marshals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Admirals of the Fleet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Full Generals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Full Admirals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Grand Chamberlain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Vice-President of the Privy Council.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Privy Councillors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Holders of 1st class Order of the Rising Sun and Paulownia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Princes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Holders of 1st class Order of the Rising Sun.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Holders of 1st class Order of the Sacred Treasure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Grand Master of Ceremonies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Grand Master of Ritualist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Lord Steward to the Empress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>President of the Administrative Litigation Court.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Civil and Military Officers of 1st grade Higher Service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Marquises.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Civil and Military Officers of 2nd grade Higher Service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Lords in Walting of Jukō Hall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Lords in Waiting of Kinkei Hall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Holders of 2nd class Order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Viscounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Holders of 3rd class Order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Barons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Printed in two columns, read left column then right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>'Precedent' (title), 'Walting' and 'Ritualist' as printed. Jukō and Kinkei printed in italics.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Principal Officials of the Imperial Household Dept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 27, 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n94/mode/1up, https://archive.org/details/japan-year-book-1910/page/n95/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Holder(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Minister</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Prince T. Iwakura</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Vice-Minister</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Visc. Watanabe</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Imperial Treasury</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>J. Yoshida, S. Sakamoto</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Imperial Archives</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>E. Yamaguchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Imperial Cookery</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Count K. Kagawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Police Affairs</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>T. Ogasawara</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dr. T. Katayama</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Gardening</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Vis. Fukuha</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Imperial Mews.</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Vis. Fujinami</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Imperial Forest Bureau</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>C. Wa[illegible]abe Visc. Y. Sasaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Peerage Bureau</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Marquis. M. Kuga, S. Obara</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Medical Affairs</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Baron. Dr. Oka; Baron T. Komeda</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Supplies and Purchase</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>S. Nagasaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Privy Seals</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Marq. Tokudaiji, T. Matano</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Board of Ceremonies</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Holder(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Grand Master of Ceremonies</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Count U. Toda</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Vice-Grand Master</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>H. Ito</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>S. Nagasaki; Marquis. Kido; R. Niwa; K. Yamanouchi; Vis. Fukuha; Y. Yoshida; M. Ichiki; Vis. [illegible]aba; Count Mayeda</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Court Councillors</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Baron S. Osaki, C. Nabeshima, M. Funakoshi, Baron M. Katori, Major-Gen. M. Sato, Vis. Takatsuji, Baron Dr. Ikeda, Vis. Fujinami, S. Nagasaki, Baron. Y. Sonoda, Marq. T. Nakayama, Prince Nijo, Marquis Kido, Prof. Y. Hozumi, Prof. K. Okano, Y. Okuda, S. Hirayama, Vis. Higashisono, Vis. Hojo, K. Maruo. Major-Gen. S. Tauchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Board of Chamberlains</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Holder(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Grand Chamberlain</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Marquis. S. Tokudaiji</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Vice-Grand Chamberlain</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Prince T. Iwakura</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Chamberlains</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Baron T. Komeda; Viscount M. Higashizono; Viscount U. Hōjō; Y. Hineno; S. Hinonishi; K. [illegible]; S. Shimizutani</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Aide-de-Camp. to H. I.M.</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>General Baron Nakamura; Rear-Adm. Baron Nishi</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>The Empress' Household</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Holder(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Viscount Kagawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>The Crown Prince's Household</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Holder(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Lieut.-General Baron Muraki</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Grand Chamberlain</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Prince S. Ichijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Chief Aide-de-Camp to the Crown [Prince]</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Lieut.-General Baron Muraki</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Printed as run-on text ('Office, Name; Office, Name; …'), split here into Office / Holder(s); names are in italics. Continues from p. 27 onto p. 28 with sub-headings Board of Ceremonies, Board of Chamberlains, The Empress' Household, The Crown Prince's Household.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Italic w often looks like 'u' in the scan: printed forms appear as 'Kagaua', 'Ogasauara', 'Iuakura' (twice), 'Kagaua' (Empress' Household); transcribed Kagawa, Ogasawara, Iwakura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>'Ka'ayama' (broken t) transcribed Katayama; 'Sakamoto' has a broken t.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Imperial Forest Bureau: 'C. Wa?a?abe' — letters broken, marked [illegible]; no punctuation visible between 'C. Wa…abe' and 'Visc. Y. Sasaki'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Medical Affairs: printed 'Baron. Dr. Oka;' at foot of p. 27, then 'Baron T. Komeda;' at top of p. 28 before 'Supplies and Purchase'; both kept under Medical Affairs as the layout gives no other office.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Board of Ceremonies Members: 'Vis. ?aba' first letter(s) broken, marked [illegible]. Board of Chamberlains: 'K. ??ewahire' unreadable, marked [illegible].</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Crown Prince's Household: 'Princ S. Ichijo' and 'Chief Aide-de-Camp to the Crown Lieut.-General Baron Muraki' printed so (line ends with a stray 'e'); '[Prince]' supplied in the office label.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" location="'Contents'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Court Ladies</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Imperial Court · printed pp. 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ladies on service at the Court and their official rank are as follows:—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Scan: https://archive.org/details/japan-year-book-1910/page/n95/mode/1up</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>← Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>"Tenji,"</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Takakura Toshi-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>"</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yanagiwara Ai-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>"Gon Tenji,"</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Chikusa To-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>" "</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ogura Fumi-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>" "</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sone Yasu-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>" "</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Anekoji Yoshi-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>" " (acting)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nishi-itsutsuji Sho-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>"Shoji"</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mibu Hiro-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>"</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Koike Michi-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>" (acting)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Nakayama Ei-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>"</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kinoshita Han-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>"Gon Shoji"</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Yobu Kine-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>" "</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Kitajima Ito-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>" "</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tsumori Yoshi-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>" "</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Awadaguchi Ayu-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>" " (acting)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kagawa Shic-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>" "</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Hirotori Kun-ko</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Footnotes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Besides the above there are eight ladies of "Myobu" rank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Transcriber's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Rank names printed in quotation marks; ditto marks (") repeat the rank above and are kept as printed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Names in italics. 'Yanagiwara' and 'Kagawa' printed with an italic w that looks like 'u' ('Yanagiuara', 'Kagaua').</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>'Yobu Kine-ko', 'Shic-ko' and 'Hirotori' as they appear in the scan (letters partly broken: 'Yc bu', 'Hiro'ori').</t>
         </is>
       </c>
     </row>

</xml_diff>